<commit_message>
Mark Alejandra as Pagado (.385)
</commit_message>
<xml_diff>
--- a/Cuentas Almuerzo con Quena.xlsx
+++ b/Cuentas Almuerzo con Quena.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,11 +59,17 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="001E3A8A"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -86,6 +92,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FEE2E2"/>
         <bgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
     <fill>
@@ -127,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -154,11 +166,14 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1261,9 +1276,9 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H3" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>Pagado</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1303,7 @@
       <c r="E4" s="7" t="n">
         <v>59230</v>
       </c>
-      <c r="F4" s="16">
+      <c r="F4" s="17">
         <f>E4-D4</f>
         <v/>
       </c>
@@ -1297,7 +1312,7 @@
           <t>Organizador (Recauda $53.845)</t>
         </is>
       </c>
-      <c r="H4" s="17" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>Organizador</t>
         </is>
@@ -1430,7 +1445,7 @@
         <f>SUM(E2:E7)</f>
         <v/>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="19">
         <f>SUMIF(G2:G7, "Transfiere a Ignacio", F2:F7)</f>
         <v/>
       </c>

</xml_diff>